<commit_message>
Adjustments to data sheets
</commit_message>
<xml_diff>
--- a/reductions-lit/data/acidification_dat_extra.xlsx
+++ b/reductions-lit/data/acidification_dat_extra.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au583430_uni_au_dk/Documents/Documents/GitHub/GD-NH3/reductions/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au583430_uni_au_dk/Documents/Documents/GitHub/GD-NH3/reductions-lit/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="409" documentId="8_{35EDC6DB-B444-4E75-9EC7-B91B9DC064D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{065AE67C-0A4B-4D0C-A35A-119D2959127F}"/>
+  <xr:revisionPtr revIDLastSave="434" documentId="8_{35EDC6DB-B444-4E75-9EC7-B91B9DC064D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52DA6C5C-94D3-4450-9C0E-F11B8AB5DA64}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-45" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Acidification_NH3_reduction_dat" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="92">
   <si>
     <t>Untreated</t>
   </si>
@@ -174,9 +174,6 @@
     <t>r</t>
   </si>
   <si>
-    <t>Huijsmans et al. (2015)</t>
-  </si>
-  <si>
     <t>Kvæg</t>
   </si>
   <si>
@@ -210,9 +207,6 @@
     <t>IHF</t>
   </si>
   <si>
-    <t>Bussink et al. (1994)</t>
-  </si>
-  <si>
     <t>before field</t>
   </si>
   <si>
@@ -291,9 +285,6 @@
     <t>WT10</t>
   </si>
   <si>
-    <t>Stevens et al. (1992)</t>
-  </si>
-  <si>
     <t>kgN/ha</t>
   </si>
   <si>
@@ -303,10 +294,22 @@
     <t>ee.a</t>
   </si>
   <si>
-    <t>Pain et al. (1990)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Studies not in the lit_dat, most of them because they are from before 2012 </t>
+  </si>
+  <si>
+    <t>Pain et al., 1990</t>
+  </si>
+  <si>
+    <t>Stevens et al., 1992</t>
+  </si>
+  <si>
+    <t>Bussink et al., 1994</t>
+  </si>
+  <si>
+    <t>Nyord, 2013</t>
+  </si>
+  <si>
+    <t>Huijsmans et al., 2015</t>
   </si>
 </sst>
 </file>
@@ -1228,10 +1231,10 @@
         <v>44</v>
       </c>
       <c r="V1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="W1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="X1" t="s">
         <v>45</v>
@@ -1239,31 +1242,31 @@
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="B2">
         <v>101</v>
       </c>
       <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
         <v>47</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>48</v>
-      </c>
-      <c r="E2" t="s">
-        <v>49</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
       <c r="G2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H2" t="s">
         <v>50</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>51</v>
-      </c>
-      <c r="I2" t="s">
-        <v>52</v>
       </c>
       <c r="J2">
         <v>23.5</v>
@@ -1301,31 +1304,31 @@
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="B3">
         <v>101</v>
       </c>
       <c r="C3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" t="s">
         <v>47</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>48</v>
-      </c>
-      <c r="E3" t="s">
-        <v>49</v>
       </c>
       <c r="F3">
         <v>4</v>
       </c>
       <c r="G3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" t="s">
         <v>50</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>51</v>
-      </c>
-      <c r="I3" t="s">
-        <v>52</v>
       </c>
       <c r="J3">
         <v>23.5</v>
@@ -1363,31 +1366,31 @@
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="B4">
         <v>101</v>
       </c>
       <c r="C4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" t="s">
         <v>47</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>48</v>
-      </c>
-      <c r="E4" t="s">
-        <v>49</v>
       </c>
       <c r="F4">
         <v>2</v>
       </c>
       <c r="G4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H4" t="s">
         <v>50</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>51</v>
-      </c>
-      <c r="I4" t="s">
-        <v>52</v>
       </c>
       <c r="J4">
         <v>21.3</v>
@@ -1425,31 +1428,31 @@
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="B5">
         <v>101</v>
       </c>
       <c r="C5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" t="s">
         <v>47</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>48</v>
-      </c>
-      <c r="E5" t="s">
-        <v>49</v>
       </c>
       <c r="F5">
         <v>4</v>
       </c>
       <c r="G5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5" t="s">
         <v>50</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>51</v>
-      </c>
-      <c r="I5" t="s">
-        <v>52</v>
       </c>
       <c r="J5">
         <v>21.3</v>
@@ -1487,31 +1490,31 @@
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="B6">
         <v>101</v>
       </c>
       <c r="C6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" t="s">
         <v>47</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>48</v>
-      </c>
-      <c r="E6" t="s">
-        <v>49</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" t="s">
         <v>50</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>51</v>
-      </c>
-      <c r="I6" t="s">
-        <v>52</v>
       </c>
       <c r="J6">
         <v>21.6</v>
@@ -1549,31 +1552,31 @@
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="B7">
         <v>101</v>
       </c>
       <c r="C7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" t="s">
         <v>47</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>48</v>
-      </c>
-      <c r="E7" t="s">
-        <v>49</v>
       </c>
       <c r="F7">
         <v>4</v>
       </c>
       <c r="G7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" t="s">
         <v>50</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>51</v>
-      </c>
-      <c r="I7" t="s">
-        <v>52</v>
       </c>
       <c r="J7">
         <v>21.6</v>
@@ -1611,31 +1614,31 @@
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="B8">
         <v>101</v>
       </c>
       <c r="C8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" t="s">
         <v>47</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>48</v>
-      </c>
-      <c r="E8" t="s">
-        <v>49</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
       <c r="G8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" t="s">
         <v>50</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>51</v>
-      </c>
-      <c r="I8" t="s">
-        <v>52</v>
       </c>
       <c r="J8">
         <v>20.9</v>
@@ -1673,31 +1676,31 @@
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="B9">
         <v>101</v>
       </c>
       <c r="C9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" t="s">
         <v>47</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>48</v>
-      </c>
-      <c r="E9" t="s">
-        <v>49</v>
       </c>
       <c r="F9">
         <v>4</v>
       </c>
       <c r="G9" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" t="s">
         <v>50</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>51</v>
-      </c>
-      <c r="I9" t="s">
-        <v>52</v>
       </c>
       <c r="J9">
         <v>20.9</v>
@@ -1735,28 +1738,28 @@
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B10">
         <v>102</v>
       </c>
       <c r="C10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" t="s">
         <v>54</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" t="s">
         <v>55</v>
       </c>
-      <c r="E10" t="s">
-        <v>49</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>56</v>
       </c>
-      <c r="H10" t="s">
-        <v>57</v>
-      </c>
       <c r="I10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J10">
         <v>31.4</v>
@@ -1800,28 +1803,28 @@
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B11">
         <v>102</v>
       </c>
       <c r="C11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" t="s">
         <v>54</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" t="s">
         <v>55</v>
       </c>
-      <c r="E11" t="s">
-        <v>49</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>56</v>
       </c>
-      <c r="H11" t="s">
-        <v>57</v>
-      </c>
       <c r="I11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J11">
         <v>31.4</v>
@@ -1865,28 +1868,28 @@
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B12">
         <v>102</v>
       </c>
       <c r="C12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" t="s">
         <v>54</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" t="s">
         <v>55</v>
       </c>
-      <c r="E12" t="s">
-        <v>49</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>56</v>
       </c>
-      <c r="H12" t="s">
-        <v>57</v>
-      </c>
       <c r="I12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J12">
         <v>31.4</v>
@@ -1930,28 +1933,28 @@
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B13">
         <v>102</v>
       </c>
       <c r="C13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" t="s">
         <v>48</v>
       </c>
-      <c r="E13" t="s">
+      <c r="G13" t="s">
         <v>49</v>
       </c>
-      <c r="G13" t="s">
-        <v>50</v>
-      </c>
       <c r="H13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J13">
         <v>31.4</v>
@@ -1995,28 +1998,28 @@
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B14">
         <v>102</v>
       </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D14" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" t="s">
         <v>48</v>
       </c>
-      <c r="E14" t="s">
+      <c r="G14" t="s">
         <v>49</v>
       </c>
-      <c r="G14" t="s">
-        <v>50</v>
-      </c>
       <c r="H14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J14">
         <v>31.4</v>
@@ -2060,28 +2063,28 @@
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B15">
         <v>102</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" t="s">
         <v>48</v>
       </c>
-      <c r="E15" t="s">
+      <c r="G15" t="s">
         <v>49</v>
       </c>
-      <c r="G15" t="s">
-        <v>50</v>
-      </c>
       <c r="H15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J15">
         <v>31.4</v>
@@ -2125,28 +2128,28 @@
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B16">
         <v>102</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D16" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" t="s">
         <v>48</v>
       </c>
-      <c r="E16" t="s">
+      <c r="G16" t="s">
         <v>49</v>
       </c>
-      <c r="G16" t="s">
-        <v>50</v>
-      </c>
       <c r="H16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J16">
         <v>31.4</v>
@@ -2190,28 +2193,28 @@
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B17">
         <v>102</v>
       </c>
       <c r="C17" t="s">
+        <v>53</v>
+      </c>
+      <c r="D17" t="s">
         <v>54</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
+        <v>48</v>
+      </c>
+      <c r="G17" t="s">
         <v>55</v>
       </c>
-      <c r="E17" t="s">
-        <v>49</v>
-      </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>56</v>
       </c>
-      <c r="H17" t="s">
-        <v>57</v>
-      </c>
       <c r="I17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J17">
         <v>31.4</v>
@@ -2255,28 +2258,28 @@
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B18">
         <v>102</v>
       </c>
       <c r="C18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18" t="s">
         <v>54</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
+        <v>48</v>
+      </c>
+      <c r="G18" t="s">
         <v>55</v>
       </c>
-      <c r="E18" t="s">
-        <v>49</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>56</v>
       </c>
-      <c r="H18" t="s">
-        <v>57</v>
-      </c>
       <c r="I18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J18">
         <v>31.4</v>
@@ -2320,28 +2323,28 @@
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B19">
         <v>102</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D19" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" t="s">
         <v>48</v>
       </c>
-      <c r="E19" t="s">
+      <c r="G19" t="s">
         <v>49</v>
       </c>
-      <c r="G19" t="s">
-        <v>50</v>
-      </c>
       <c r="H19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J19">
         <v>31.4</v>
@@ -2385,28 +2388,28 @@
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B20">
         <v>102</v>
       </c>
       <c r="C20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" t="s">
         <v>48</v>
       </c>
-      <c r="E20" t="s">
+      <c r="G20" t="s">
         <v>49</v>
       </c>
-      <c r="G20" t="s">
-        <v>50</v>
-      </c>
       <c r="H20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J20">
         <v>31.4</v>
@@ -2450,28 +2453,28 @@
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="B21">
         <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D21" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" t="s">
         <v>48</v>
       </c>
-      <c r="E21" t="s">
+      <c r="G21" t="s">
         <v>49</v>
       </c>
-      <c r="G21" t="s">
-        <v>50</v>
-      </c>
       <c r="H21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J21">
         <v>31.4</v>
@@ -2515,28 +2518,28 @@
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B22">
         <v>102</v>
       </c>
       <c r="C22" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" t="s">
         <v>54</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
+        <v>48</v>
+      </c>
+      <c r="G22" t="s">
         <v>55</v>
       </c>
-      <c r="E22" t="s">
-        <v>49</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>56</v>
       </c>
-      <c r="H22" t="s">
-        <v>57</v>
-      </c>
       <c r="I22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J22">
         <v>31.4</v>
@@ -2580,25 +2583,25 @@
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B23">
         <v>104</v>
       </c>
       <c r="C23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D23" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" t="s">
+        <v>58</v>
+      </c>
+      <c r="H23" t="s">
         <v>59</v>
       </c>
-      <c r="E23" t="s">
-        <v>60</v>
-      </c>
-      <c r="H23" t="s">
-        <v>61</v>
-      </c>
       <c r="I23" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J23">
         <v>10</v>
@@ -2633,25 +2636,25 @@
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B24">
         <v>104</v>
       </c>
       <c r="C24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D24" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E24" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H24" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I24" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J24">
         <v>10</v>
@@ -2686,25 +2689,25 @@
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B25">
         <v>104</v>
       </c>
       <c r="C25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D25" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E25" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H25" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I25" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J25">
         <v>6.5</v>
@@ -2745,25 +2748,25 @@
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B26">
         <v>104</v>
       </c>
       <c r="C26" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D26" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E26" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H26" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I26" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J26">
         <v>10.199999999999999</v>
@@ -2804,25 +2807,25 @@
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B27">
         <v>104</v>
       </c>
       <c r="C27" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D27" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E27" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H27" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I27" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J27">
         <v>9.8000000000000007</v>
@@ -2863,25 +2866,25 @@
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B28">
         <v>104</v>
       </c>
       <c r="C28" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D28" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E28" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I28" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J28">
         <v>9.9</v>
@@ -2922,25 +2925,25 @@
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B29">
         <v>104</v>
       </c>
       <c r="C29" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D29" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E29" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H29" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J29">
         <v>9.8000000000000007</v>
@@ -2981,25 +2984,25 @@
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B30">
         <v>104</v>
       </c>
       <c r="C30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D30" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E30" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H30" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I30" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J30">
         <v>12.7</v>
@@ -3040,25 +3043,25 @@
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B31">
         <v>104</v>
       </c>
       <c r="C31" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D31" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E31" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H31" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I31" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J31">
         <v>9.6</v>
@@ -3099,25 +3102,25 @@
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B32">
         <v>104</v>
       </c>
       <c r="C32" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D32" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E32" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H32" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I32" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J32">
         <v>8.6999999999999993</v>
@@ -3158,25 +3161,25 @@
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B33">
         <v>104</v>
       </c>
       <c r="C33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D33" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E33" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H33" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I33" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J33">
         <v>9.8000000000000007</v>
@@ -3217,25 +3220,25 @@
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B34">
         <v>104</v>
       </c>
       <c r="C34" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D34" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E34" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H34" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I34" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J34">
         <v>9.8000000000000007</v>
@@ -3276,25 +3279,25 @@
     </row>
     <row r="35" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B35">
         <v>104</v>
       </c>
       <c r="C35" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D35" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E35" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I35" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J35">
         <v>9.8000000000000007</v>
@@ -3335,25 +3338,25 @@
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B36">
         <v>104</v>
       </c>
       <c r="C36" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D36" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E36" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H36" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I36" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J36">
         <v>17.3</v>
@@ -3394,25 +3397,25 @@
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B37">
         <v>104</v>
       </c>
       <c r="C37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D37" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E37" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H37" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I37" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J37">
         <v>17.3</v>
@@ -3453,25 +3456,25 @@
     </row>
     <row r="38" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B38">
         <v>104</v>
       </c>
       <c r="C38" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D38" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E38" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H38" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I38" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J38">
         <v>17.3</v>
@@ -3512,25 +3515,25 @@
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B39">
         <v>104</v>
       </c>
       <c r="C39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D39" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E39" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H39" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I39" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J39">
         <v>11.6</v>
@@ -3571,25 +3574,25 @@
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B40">
         <v>104</v>
       </c>
       <c r="C40" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D40" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E40" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H40" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J40">
         <v>11.6</v>
@@ -3630,25 +3633,25 @@
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B41">
         <v>104</v>
       </c>
       <c r="C41" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D41" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E41" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H41" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I41" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J41">
         <v>11.6</v>
@@ -3689,25 +3692,25 @@
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B42">
         <v>104</v>
       </c>
       <c r="C42" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D42" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E42" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H42" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I42" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J42">
         <v>14.8</v>
@@ -3745,25 +3748,25 @@
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B43">
         <v>104</v>
       </c>
       <c r="C43" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D43" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E43" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H43" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I43" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J43">
         <v>10.199999999999999</v>
@@ -3801,25 +3804,25 @@
     </row>
     <row r="44" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B44">
         <v>104</v>
       </c>
       <c r="C44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D44" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E44" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H44" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="I44" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J44">
         <v>22</v>
@@ -3857,25 +3860,25 @@
     </row>
     <row r="45" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B45">
         <v>104</v>
       </c>
       <c r="C45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D45" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E45" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H45" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I45" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J45">
         <v>22</v>
@@ -3913,25 +3916,25 @@
     </row>
     <row r="46" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B46">
         <v>104</v>
       </c>
       <c r="C46" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D46" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E46" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H46" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I46" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J46">
         <v>30</v>
@@ -3969,25 +3972,25 @@
     </row>
     <row r="47" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B47">
         <v>104</v>
       </c>
       <c r="C47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D47" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E47" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H47" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I47" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J47">
         <v>22</v>
@@ -4025,25 +4028,25 @@
     </row>
     <row r="48" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B48">
         <v>104</v>
       </c>
       <c r="C48" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D48" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E48" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H48" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I48" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J48">
         <v>30</v>
@@ -4081,25 +4084,25 @@
     </row>
     <row r="49" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B49">
         <v>104</v>
       </c>
       <c r="C49" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D49" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E49" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H49" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="I49" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J49">
         <v>30</v>
@@ -4137,25 +4140,25 @@
     </row>
     <row r="50" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B50">
         <v>104</v>
       </c>
       <c r="C50" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D50" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E50" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H50" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I50" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J50">
         <v>30</v>
@@ -4193,25 +4196,25 @@
     </row>
     <row r="51" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="B51">
         <v>104</v>
       </c>
       <c r="C51" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D51" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E51" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H51" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I51" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J51">
         <v>30</v>
@@ -4249,19 +4252,19 @@
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B52">
         <v>114</v>
       </c>
       <c r="D52" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E52" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I52" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K52">
         <v>7.5</v>
@@ -4282,19 +4285,19 @@
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B53">
         <v>114</v>
       </c>
       <c r="D53" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E53" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I53" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K53">
         <v>7.5</v>
@@ -4315,19 +4318,19 @@
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B54">
         <v>114</v>
       </c>
       <c r="D54" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E54" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I54" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K54">
         <v>7.5</v>
@@ -4348,19 +4351,19 @@
     </row>
     <row r="55" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B55">
         <v>114</v>
       </c>
       <c r="D55" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E55" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I55" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K55">
         <v>7.5</v>
@@ -4381,19 +4384,19 @@
     </row>
     <row r="56" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B56">
         <v>114</v>
       </c>
       <c r="D56" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E56" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I56" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K56">
         <v>7.5</v>
@@ -4414,19 +4417,19 @@
     </row>
     <row r="57" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B57">
         <v>114</v>
       </c>
       <c r="D57" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E57" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I57" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K57">
         <v>7.5</v>
@@ -4447,19 +4450,19 @@
     </row>
     <row r="58" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B58">
         <v>114</v>
       </c>
       <c r="D58" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E58" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I58" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K58">
         <v>7.5</v>
@@ -4480,19 +4483,19 @@
     </row>
     <row r="59" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B59">
         <v>114</v>
       </c>
       <c r="D59" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E59" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I59" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K59">
         <v>7.5</v>
@@ -4513,19 +4516,19 @@
     </row>
     <row r="60" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B60">
         <v>114</v>
       </c>
       <c r="D60" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E60" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I60" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K60">
         <v>7.5</v>
@@ -4546,19 +4549,19 @@
     </row>
     <row r="61" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B61">
         <v>114</v>
       </c>
       <c r="D61" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E61" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I61" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K61">
         <v>7.5</v>
@@ -4579,19 +4582,19 @@
     </row>
     <row r="62" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B62">
         <v>114</v>
       </c>
       <c r="D62" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E62" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I62" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K62">
         <v>7.5</v>
@@ -4612,19 +4615,19 @@
     </row>
     <row r="63" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B63">
         <v>114</v>
       </c>
       <c r="D63" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E63" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I63" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K63">
         <v>7.5</v>
@@ -4645,19 +4648,19 @@
     </row>
     <row r="64" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B64">
         <v>114</v>
       </c>
       <c r="D64" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E64" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I64" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K64">
         <v>7.5</v>
@@ -4678,19 +4681,19 @@
     </row>
     <row r="65" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B65">
         <v>114</v>
       </c>
       <c r="D65" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E65" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I65" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K65">
         <v>7.5</v>
@@ -4711,19 +4714,19 @@
     </row>
     <row r="66" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B66">
         <v>114</v>
       </c>
       <c r="D66" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E66" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I66" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K66">
         <v>7.5</v>
@@ -4744,19 +4747,19 @@
     </row>
     <row r="67" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B67">
         <v>114</v>
       </c>
       <c r="D67" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E67" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I67" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K67">
         <v>7.5</v>
@@ -4777,19 +4780,19 @@
     </row>
     <row r="68" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B68">
         <v>114</v>
       </c>
       <c r="D68" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E68" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I68" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K68">
         <v>7.5</v>
@@ -4810,19 +4813,19 @@
     </row>
     <row r="69" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B69">
         <v>114</v>
       </c>
       <c r="D69" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E69" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I69" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K69">
         <v>7.5</v>
@@ -4843,19 +4846,19 @@
     </row>
     <row r="70" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B70">
         <v>114</v>
       </c>
       <c r="D70" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E70" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I70" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K70">
         <v>7.9</v>
@@ -4875,19 +4878,19 @@
     </row>
     <row r="71" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B71">
         <v>114</v>
       </c>
       <c r="D71" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E71" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I71" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K71">
         <v>7.9</v>
@@ -4907,19 +4910,19 @@
     </row>
     <row r="72" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B72">
         <v>114</v>
       </c>
       <c r="D72" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E72" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I72" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K72">
         <v>7.9</v>
@@ -4939,19 +4942,19 @@
     </row>
     <row r="73" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B73">
         <v>114</v>
       </c>
       <c r="D73" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E73" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I73" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K73">
         <v>7.9</v>
@@ -4971,19 +4974,19 @@
     </row>
     <row r="74" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B74">
         <v>114</v>
       </c>
       <c r="D74" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E74" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I74" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K74">
         <v>7.9</v>
@@ -5003,19 +5006,19 @@
     </row>
     <row r="75" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B75">
         <v>114</v>
       </c>
       <c r="D75" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E75" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I75" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K75">
         <v>7.9</v>
@@ -5035,19 +5038,19 @@
     </row>
     <row r="76" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B76">
         <v>114</v>
       </c>
       <c r="D76" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E76" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I76" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K76">
         <v>7.9</v>
@@ -5067,19 +5070,19 @@
     </row>
     <row r="77" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B77">
         <v>114</v>
       </c>
       <c r="D77" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E77" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I77" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K77">
         <v>7.9</v>
@@ -5099,19 +5102,19 @@
     </row>
     <row r="78" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B78">
         <v>114</v>
       </c>
       <c r="D78" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E78" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I78" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K78">
         <v>7.9</v>
@@ -5131,19 +5134,19 @@
     </row>
     <row r="79" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B79">
         <v>114</v>
       </c>
       <c r="D79" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E79" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I79" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K79">
         <v>7.9</v>
@@ -5163,19 +5166,19 @@
     </row>
     <row r="80" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B80">
         <v>114</v>
       </c>
       <c r="D80" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E80" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I80" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K80">
         <v>7.9</v>
@@ -5195,19 +5198,19 @@
     </row>
     <row r="81" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B81">
         <v>114</v>
       </c>
       <c r="D81" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E81" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I81" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K81">
         <v>7.9</v>
@@ -5227,19 +5230,19 @@
     </row>
     <row r="82" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B82">
         <v>114</v>
       </c>
       <c r="D82" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E82" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I82" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K82">
         <v>7.9</v>
@@ -5259,19 +5262,19 @@
     </row>
     <row r="83" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B83">
         <v>114</v>
       </c>
       <c r="D83" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E83" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I83" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K83">
         <v>7.9</v>
@@ -5291,19 +5294,19 @@
     </row>
     <row r="84" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B84">
         <v>114</v>
       </c>
       <c r="D84" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E84" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I84" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K84">
         <v>7.9</v>
@@ -5323,19 +5326,19 @@
     </row>
     <row r="85" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B85">
         <v>114</v>
       </c>
       <c r="D85" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E85" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I85" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K85">
         <v>7.9</v>
@@ -5355,19 +5358,19 @@
     </row>
     <row r="86" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B86">
         <v>114</v>
       </c>
       <c r="D86" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E86" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I86" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K86">
         <v>7.9</v>
@@ -5387,19 +5390,19 @@
     </row>
     <row r="87" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B87">
         <v>114</v>
       </c>
       <c r="D87" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E87" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I87" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K87">
         <v>7.9</v>
@@ -5419,19 +5422,19 @@
     </row>
     <row r="88" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B88">
         <v>114</v>
       </c>
       <c r="D88" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E88" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I88" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K88">
         <v>7.9</v>
@@ -5451,19 +5454,19 @@
     </row>
     <row r="89" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B89">
         <v>114</v>
       </c>
       <c r="D89" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E89" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="I89" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K89">
         <v>7.9</v>
@@ -5483,19 +5486,19 @@
     </row>
     <row r="90" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B90">
         <v>115</v>
       </c>
       <c r="D90" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E90" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I90" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K90">
         <v>7.4</v>
@@ -5515,19 +5518,19 @@
     </row>
     <row r="91" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B91">
         <v>115</v>
       </c>
       <c r="D91" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E91" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I91" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K91">
         <v>7.4</v>
@@ -5547,19 +5550,19 @@
     </row>
     <row r="92" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B92">
         <v>115</v>
       </c>
       <c r="D92" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E92" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I92" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K92">
         <v>7.3</v>
@@ -5579,19 +5582,19 @@
     </row>
     <row r="93" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B93">
         <v>115</v>
       </c>
       <c r="D93" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E93" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I93" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K93">
         <v>7.3</v>
@@ -5761,10 +5764,10 @@
         <v>24</v>
       </c>
       <c r="V3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="W3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="X3" t="s">
         <v>25</v>
@@ -5835,10 +5838,10 @@
         <v>44</v>
       </c>
       <c r="V4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="W4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="X4" t="s">
         <v>45</v>
@@ -5846,7 +5849,7 @@
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
minor adjustments to data sheets
</commit_message>
<xml_diff>
--- a/reductions-lit/data/acidification_dat_extra.xlsx
+++ b/reductions-lit/data/acidification_dat_extra.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au583430_uni_au_dk/Documents/Documents/GitHub/GD-NH3/reductions-lit/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="434" documentId="8_{35EDC6DB-B444-4E75-9EC7-B91B9DC064D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52DA6C5C-94D3-4450-9C0E-F11B8AB5DA64}"/>
+  <xr:revisionPtr revIDLastSave="435" documentId="8_{35EDC6DB-B444-4E75-9EC7-B91B9DC064D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{511A7B62-0C87-4815-8D34-D4ACF218E72E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="91">
   <si>
     <t>Untreated</t>
   </si>
@@ -190,9 +190,6 @@
   </si>
   <si>
     <t>band</t>
-  </si>
-  <si>
-    <t>Nyord (2013)</t>
   </si>
   <si>
     <t>Svin</t>
@@ -1231,10 +1228,10 @@
         <v>44</v>
       </c>
       <c r="V1" t="s">
+        <v>83</v>
+      </c>
+      <c r="W1" t="s">
         <v>84</v>
-      </c>
-      <c r="W1" t="s">
-        <v>85</v>
       </c>
       <c r="X1" t="s">
         <v>45</v>
@@ -1242,7 +1239,7 @@
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B2">
         <v>101</v>
@@ -1304,7 +1301,7 @@
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B3">
         <v>101</v>
@@ -1366,7 +1363,7 @@
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B4">
         <v>101</v>
@@ -1428,7 +1425,7 @@
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B5">
         <v>101</v>
@@ -1490,7 +1487,7 @@
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B6">
         <v>101</v>
@@ -1552,7 +1549,7 @@
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B7">
         <v>101</v>
@@ -1614,7 +1611,7 @@
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B8">
         <v>101</v>
@@ -1676,7 +1673,7 @@
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B9">
         <v>101</v>
@@ -1738,25 +1735,25 @@
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B10">
         <v>102</v>
       </c>
       <c r="C10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" t="s">
         <v>53</v>
-      </c>
-      <c r="D10" t="s">
-        <v>54</v>
       </c>
       <c r="E10" t="s">
         <v>48</v>
       </c>
       <c r="G10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" t="s">
         <v>55</v>
-      </c>
-      <c r="H10" t="s">
-        <v>56</v>
       </c>
       <c r="I10" t="s">
         <v>51</v>
@@ -1803,25 +1800,25 @@
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B11">
         <v>102</v>
       </c>
       <c r="C11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" t="s">
         <v>53</v>
-      </c>
-      <c r="D11" t="s">
-        <v>54</v>
       </c>
       <c r="E11" t="s">
         <v>48</v>
       </c>
       <c r="G11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H11" t="s">
         <v>55</v>
-      </c>
-      <c r="H11" t="s">
-        <v>56</v>
       </c>
       <c r="I11" t="s">
         <v>51</v>
@@ -1868,25 +1865,25 @@
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B12">
         <v>102</v>
       </c>
       <c r="C12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" t="s">
         <v>53</v>
-      </c>
-      <c r="D12" t="s">
-        <v>54</v>
       </c>
       <c r="E12" t="s">
         <v>48</v>
       </c>
       <c r="G12" t="s">
+        <v>54</v>
+      </c>
+      <c r="H12" t="s">
         <v>55</v>
-      </c>
-      <c r="H12" t="s">
-        <v>56</v>
       </c>
       <c r="I12" t="s">
         <v>51</v>
@@ -1933,13 +1930,13 @@
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B13">
         <v>102</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D13" t="s">
         <v>47</v>
@@ -1951,7 +1948,7 @@
         <v>49</v>
       </c>
       <c r="H13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I13" t="s">
         <v>51</v>
@@ -1998,13 +1995,13 @@
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B14">
         <v>102</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D14" t="s">
         <v>47</v>
@@ -2016,7 +2013,7 @@
         <v>49</v>
       </c>
       <c r="H14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I14" t="s">
         <v>51</v>
@@ -2063,13 +2060,13 @@
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B15">
         <v>102</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D15" t="s">
         <v>47</v>
@@ -2081,7 +2078,7 @@
         <v>49</v>
       </c>
       <c r="H15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I15" t="s">
         <v>51</v>
@@ -2128,13 +2125,13 @@
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B16">
         <v>102</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16" t="s">
         <v>47</v>
@@ -2146,7 +2143,7 @@
         <v>49</v>
       </c>
       <c r="H16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I16" t="s">
         <v>51</v>
@@ -2193,25 +2190,25 @@
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B17">
         <v>102</v>
       </c>
       <c r="C17" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" t="s">
         <v>53</v>
-      </c>
-      <c r="D17" t="s">
-        <v>54</v>
       </c>
       <c r="E17" t="s">
         <v>48</v>
       </c>
       <c r="G17" t="s">
+        <v>54</v>
+      </c>
+      <c r="H17" t="s">
         <v>55</v>
-      </c>
-      <c r="H17" t="s">
-        <v>56</v>
       </c>
       <c r="I17" t="s">
         <v>51</v>
@@ -2258,25 +2255,25 @@
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B18">
         <v>102</v>
       </c>
       <c r="C18" t="s">
+        <v>52</v>
+      </c>
+      <c r="D18" t="s">
         <v>53</v>
-      </c>
-      <c r="D18" t="s">
-        <v>54</v>
       </c>
       <c r="E18" t="s">
         <v>48</v>
       </c>
       <c r="G18" t="s">
+        <v>54</v>
+      </c>
+      <c r="H18" t="s">
         <v>55</v>
-      </c>
-      <c r="H18" t="s">
-        <v>56</v>
       </c>
       <c r="I18" t="s">
         <v>51</v>
@@ -2323,13 +2320,13 @@
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B19">
         <v>102</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D19" t="s">
         <v>47</v>
@@ -2341,7 +2338,7 @@
         <v>49</v>
       </c>
       <c r="H19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I19" t="s">
         <v>51</v>
@@ -2388,13 +2385,13 @@
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B20">
         <v>102</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D20" t="s">
         <v>47</v>
@@ -2406,7 +2403,7 @@
         <v>49</v>
       </c>
       <c r="H20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I20" t="s">
         <v>51</v>
@@ -2453,13 +2450,13 @@
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B21">
         <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D21" t="s">
         <v>47</v>
@@ -2471,7 +2468,7 @@
         <v>49</v>
       </c>
       <c r="H21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I21" t="s">
         <v>51</v>
@@ -2518,25 +2515,25 @@
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="B22">
         <v>102</v>
       </c>
       <c r="C22" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" t="s">
         <v>53</v>
-      </c>
-      <c r="D22" t="s">
-        <v>54</v>
       </c>
       <c r="E22" t="s">
         <v>48</v>
       </c>
       <c r="G22" t="s">
+        <v>54</v>
+      </c>
+      <c r="H22" t="s">
         <v>55</v>
-      </c>
-      <c r="H22" t="s">
-        <v>56</v>
       </c>
       <c r="I22" t="s">
         <v>51</v>
@@ -2583,7 +2580,7 @@
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B23">
         <v>104</v>
@@ -2592,16 +2589,16 @@
         <v>46</v>
       </c>
       <c r="D23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E23" t="s">
         <v>57</v>
       </c>
-      <c r="E23" t="s">
+      <c r="H23" t="s">
         <v>58</v>
       </c>
-      <c r="H23" t="s">
-        <v>59</v>
-      </c>
       <c r="I23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J23">
         <v>10</v>
@@ -2636,7 +2633,7 @@
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B24">
         <v>104</v>
@@ -2645,16 +2642,16 @@
         <v>46</v>
       </c>
       <c r="D24" t="s">
+        <v>56</v>
+      </c>
+      <c r="E24" t="s">
         <v>57</v>
       </c>
-      <c r="E24" t="s">
-        <v>58</v>
-      </c>
       <c r="H24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J24">
         <v>10</v>
@@ -2689,7 +2686,7 @@
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B25">
         <v>104</v>
@@ -2698,16 +2695,16 @@
         <v>46</v>
       </c>
       <c r="D25" t="s">
+        <v>56</v>
+      </c>
+      <c r="E25" t="s">
         <v>57</v>
       </c>
-      <c r="E25" t="s">
-        <v>58</v>
-      </c>
       <c r="H25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J25">
         <v>6.5</v>
@@ -2748,7 +2745,7 @@
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B26">
         <v>104</v>
@@ -2757,16 +2754,16 @@
         <v>46</v>
       </c>
       <c r="D26" t="s">
+        <v>56</v>
+      </c>
+      <c r="E26" t="s">
         <v>57</v>
       </c>
-      <c r="E26" t="s">
-        <v>58</v>
-      </c>
       <c r="H26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J26">
         <v>10.199999999999999</v>
@@ -2807,7 +2804,7 @@
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B27">
         <v>104</v>
@@ -2816,16 +2813,16 @@
         <v>46</v>
       </c>
       <c r="D27" t="s">
+        <v>56</v>
+      </c>
+      <c r="E27" t="s">
         <v>57</v>
       </c>
-      <c r="E27" t="s">
-        <v>58</v>
-      </c>
       <c r="H27" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J27">
         <v>9.8000000000000007</v>
@@ -2866,7 +2863,7 @@
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B28">
         <v>104</v>
@@ -2875,16 +2872,16 @@
         <v>46</v>
       </c>
       <c r="D28" t="s">
+        <v>56</v>
+      </c>
+      <c r="E28" t="s">
         <v>57</v>
       </c>
-      <c r="E28" t="s">
-        <v>58</v>
-      </c>
       <c r="H28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J28">
         <v>9.9</v>
@@ -2925,7 +2922,7 @@
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B29">
         <v>104</v>
@@ -2934,16 +2931,16 @@
         <v>46</v>
       </c>
       <c r="D29" t="s">
+        <v>56</v>
+      </c>
+      <c r="E29" t="s">
         <v>57</v>
       </c>
-      <c r="E29" t="s">
-        <v>58</v>
-      </c>
       <c r="H29" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J29">
         <v>9.8000000000000007</v>
@@ -2984,7 +2981,7 @@
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B30">
         <v>104</v>
@@ -2993,16 +2990,16 @@
         <v>46</v>
       </c>
       <c r="D30" t="s">
+        <v>56</v>
+      </c>
+      <c r="E30" t="s">
         <v>57</v>
       </c>
-      <c r="E30" t="s">
-        <v>58</v>
-      </c>
       <c r="H30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J30">
         <v>12.7</v>
@@ -3043,7 +3040,7 @@
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B31">
         <v>104</v>
@@ -3052,16 +3049,16 @@
         <v>46</v>
       </c>
       <c r="D31" t="s">
+        <v>56</v>
+      </c>
+      <c r="E31" t="s">
         <v>57</v>
       </c>
-      <c r="E31" t="s">
-        <v>58</v>
-      </c>
       <c r="H31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I31" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J31">
         <v>9.6</v>
@@ -3102,7 +3099,7 @@
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B32">
         <v>104</v>
@@ -3111,16 +3108,16 @@
         <v>46</v>
       </c>
       <c r="D32" t="s">
+        <v>56</v>
+      </c>
+      <c r="E32" t="s">
         <v>57</v>
       </c>
-      <c r="E32" t="s">
-        <v>58</v>
-      </c>
       <c r="H32" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J32">
         <v>8.6999999999999993</v>
@@ -3161,7 +3158,7 @@
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B33">
         <v>104</v>
@@ -3170,16 +3167,16 @@
         <v>46</v>
       </c>
       <c r="D33" t="s">
+        <v>56</v>
+      </c>
+      <c r="E33" t="s">
         <v>57</v>
       </c>
-      <c r="E33" t="s">
-        <v>58</v>
-      </c>
       <c r="H33" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I33" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J33">
         <v>9.8000000000000007</v>
@@ -3220,7 +3217,7 @@
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B34">
         <v>104</v>
@@ -3229,16 +3226,16 @@
         <v>46</v>
       </c>
       <c r="D34" t="s">
+        <v>56</v>
+      </c>
+      <c r="E34" t="s">
         <v>57</v>
       </c>
-      <c r="E34" t="s">
-        <v>58</v>
-      </c>
       <c r="H34" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I34" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J34">
         <v>9.8000000000000007</v>
@@ -3279,7 +3276,7 @@
     </row>
     <row r="35" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B35">
         <v>104</v>
@@ -3288,16 +3285,16 @@
         <v>46</v>
       </c>
       <c r="D35" t="s">
+        <v>56</v>
+      </c>
+      <c r="E35" t="s">
         <v>57</v>
       </c>
-      <c r="E35" t="s">
-        <v>58</v>
-      </c>
       <c r="H35" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J35">
         <v>9.8000000000000007</v>
@@ -3338,7 +3335,7 @@
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B36">
         <v>104</v>
@@ -3347,16 +3344,16 @@
         <v>46</v>
       </c>
       <c r="D36" t="s">
+        <v>56</v>
+      </c>
+      <c r="E36" t="s">
         <v>57</v>
       </c>
-      <c r="E36" t="s">
-        <v>58</v>
-      </c>
       <c r="H36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I36" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J36">
         <v>17.3</v>
@@ -3397,7 +3394,7 @@
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B37">
         <v>104</v>
@@ -3406,16 +3403,16 @@
         <v>46</v>
       </c>
       <c r="D37" t="s">
+        <v>56</v>
+      </c>
+      <c r="E37" t="s">
         <v>57</v>
       </c>
-      <c r="E37" t="s">
-        <v>58</v>
-      </c>
       <c r="H37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J37">
         <v>17.3</v>
@@ -3456,7 +3453,7 @@
     </row>
     <row r="38" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B38">
         <v>104</v>
@@ -3465,16 +3462,16 @@
         <v>46</v>
       </c>
       <c r="D38" t="s">
+        <v>56</v>
+      </c>
+      <c r="E38" t="s">
         <v>57</v>
       </c>
-      <c r="E38" t="s">
-        <v>58</v>
-      </c>
       <c r="H38" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J38">
         <v>17.3</v>
@@ -3515,7 +3512,7 @@
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B39">
         <v>104</v>
@@ -3524,16 +3521,16 @@
         <v>46</v>
       </c>
       <c r="D39" t="s">
+        <v>56</v>
+      </c>
+      <c r="E39" t="s">
         <v>57</v>
       </c>
-      <c r="E39" t="s">
-        <v>58</v>
-      </c>
       <c r="H39" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I39" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J39">
         <v>11.6</v>
@@ -3574,7 +3571,7 @@
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B40">
         <v>104</v>
@@ -3583,16 +3580,16 @@
         <v>46</v>
       </c>
       <c r="D40" t="s">
+        <v>56</v>
+      </c>
+      <c r="E40" t="s">
         <v>57</v>
       </c>
-      <c r="E40" t="s">
-        <v>58</v>
-      </c>
       <c r="H40" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I40" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J40">
         <v>11.6</v>
@@ -3633,7 +3630,7 @@
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B41">
         <v>104</v>
@@ -3642,16 +3639,16 @@
         <v>46</v>
       </c>
       <c r="D41" t="s">
+        <v>56</v>
+      </c>
+      <c r="E41" t="s">
         <v>57</v>
       </c>
-      <c r="E41" t="s">
-        <v>58</v>
-      </c>
       <c r="H41" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I41" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J41">
         <v>11.6</v>
@@ -3692,7 +3689,7 @@
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B42">
         <v>104</v>
@@ -3701,16 +3698,16 @@
         <v>46</v>
       </c>
       <c r="D42" t="s">
+        <v>56</v>
+      </c>
+      <c r="E42" t="s">
         <v>57</v>
       </c>
-      <c r="E42" t="s">
-        <v>58</v>
-      </c>
       <c r="H42" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I42" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J42">
         <v>14.8</v>
@@ -3748,7 +3745,7 @@
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B43">
         <v>104</v>
@@ -3757,16 +3754,16 @@
         <v>46</v>
       </c>
       <c r="D43" t="s">
+        <v>56</v>
+      </c>
+      <c r="E43" t="s">
         <v>57</v>
       </c>
-      <c r="E43" t="s">
-        <v>58</v>
-      </c>
       <c r="H43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J43">
         <v>10.199999999999999</v>
@@ -3804,7 +3801,7 @@
     </row>
     <row r="44" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B44">
         <v>104</v>
@@ -3813,16 +3810,16 @@
         <v>46</v>
       </c>
       <c r="D44" t="s">
+        <v>56</v>
+      </c>
+      <c r="E44" t="s">
         <v>57</v>
       </c>
-      <c r="E44" t="s">
-        <v>58</v>
-      </c>
       <c r="H44" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I44" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J44">
         <v>22</v>
@@ -3860,7 +3857,7 @@
     </row>
     <row r="45" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B45">
         <v>104</v>
@@ -3869,16 +3866,16 @@
         <v>46</v>
       </c>
       <c r="D45" t="s">
+        <v>56</v>
+      </c>
+      <c r="E45" t="s">
         <v>57</v>
       </c>
-      <c r="E45" t="s">
-        <v>58</v>
-      </c>
       <c r="H45" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I45" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J45">
         <v>22</v>
@@ -3916,7 +3913,7 @@
     </row>
     <row r="46" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B46">
         <v>104</v>
@@ -3925,16 +3922,16 @@
         <v>46</v>
       </c>
       <c r="D46" t="s">
+        <v>56</v>
+      </c>
+      <c r="E46" t="s">
         <v>57</v>
       </c>
-      <c r="E46" t="s">
-        <v>58</v>
-      </c>
       <c r="H46" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I46" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J46">
         <v>30</v>
@@ -3972,7 +3969,7 @@
     </row>
     <row r="47" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B47">
         <v>104</v>
@@ -3981,16 +3978,16 @@
         <v>46</v>
       </c>
       <c r="D47" t="s">
+        <v>56</v>
+      </c>
+      <c r="E47" t="s">
         <v>57</v>
       </c>
-      <c r="E47" t="s">
-        <v>58</v>
-      </c>
       <c r="H47" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I47" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J47">
         <v>22</v>
@@ -4028,7 +4025,7 @@
     </row>
     <row r="48" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B48">
         <v>104</v>
@@ -4037,16 +4034,16 @@
         <v>46</v>
       </c>
       <c r="D48" t="s">
+        <v>56</v>
+      </c>
+      <c r="E48" t="s">
         <v>57</v>
       </c>
-      <c r="E48" t="s">
-        <v>58</v>
-      </c>
       <c r="H48" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I48" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J48">
         <v>30</v>
@@ -4084,7 +4081,7 @@
     </row>
     <row r="49" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B49">
         <v>104</v>
@@ -4093,16 +4090,16 @@
         <v>46</v>
       </c>
       <c r="D49" t="s">
+        <v>56</v>
+      </c>
+      <c r="E49" t="s">
         <v>57</v>
       </c>
-      <c r="E49" t="s">
-        <v>58</v>
-      </c>
       <c r="H49" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I49" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J49">
         <v>30</v>
@@ -4140,7 +4137,7 @@
     </row>
     <row r="50" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B50">
         <v>104</v>
@@ -4149,16 +4146,16 @@
         <v>46</v>
       </c>
       <c r="D50" t="s">
+        <v>56</v>
+      </c>
+      <c r="E50" t="s">
         <v>57</v>
       </c>
-      <c r="E50" t="s">
-        <v>58</v>
-      </c>
       <c r="H50" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I50" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J50">
         <v>30</v>
@@ -4196,7 +4193,7 @@
     </row>
     <row r="51" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B51">
         <v>104</v>
@@ -4205,16 +4202,16 @@
         <v>46</v>
       </c>
       <c r="D51" t="s">
+        <v>56</v>
+      </c>
+      <c r="E51" t="s">
         <v>57</v>
       </c>
-      <c r="E51" t="s">
-        <v>58</v>
-      </c>
       <c r="H51" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I51" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J51">
         <v>30</v>
@@ -4252,19 +4249,19 @@
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B52">
         <v>114</v>
       </c>
       <c r="D52" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E52" t="s">
         <v>48</v>
       </c>
       <c r="I52" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K52">
         <v>7.5</v>
@@ -4285,19 +4282,19 @@
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B53">
         <v>114</v>
       </c>
       <c r="D53" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E53" t="s">
         <v>48</v>
       </c>
       <c r="I53" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K53">
         <v>7.5</v>
@@ -4318,19 +4315,19 @@
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B54">
         <v>114</v>
       </c>
       <c r="D54" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E54" t="s">
         <v>48</v>
       </c>
       <c r="I54" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K54">
         <v>7.5</v>
@@ -4351,19 +4348,19 @@
     </row>
     <row r="55" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B55">
         <v>114</v>
       </c>
       <c r="D55" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E55" t="s">
         <v>48</v>
       </c>
       <c r="I55" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K55">
         <v>7.5</v>
@@ -4384,19 +4381,19 @@
     </row>
     <row r="56" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B56">
         <v>114</v>
       </c>
       <c r="D56" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E56" t="s">
         <v>48</v>
       </c>
       <c r="I56" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K56">
         <v>7.5</v>
@@ -4417,19 +4414,19 @@
     </row>
     <row r="57" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B57">
         <v>114</v>
       </c>
       <c r="D57" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E57" t="s">
         <v>48</v>
       </c>
       <c r="I57" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K57">
         <v>7.5</v>
@@ -4450,19 +4447,19 @@
     </row>
     <row r="58" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B58">
         <v>114</v>
       </c>
       <c r="D58" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E58" t="s">
         <v>48</v>
       </c>
       <c r="I58" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K58">
         <v>7.5</v>
@@ -4483,19 +4480,19 @@
     </row>
     <row r="59" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B59">
         <v>114</v>
       </c>
       <c r="D59" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E59" t="s">
         <v>48</v>
       </c>
       <c r="I59" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K59">
         <v>7.5</v>
@@ -4516,19 +4513,19 @@
     </row>
     <row r="60" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B60">
         <v>114</v>
       </c>
       <c r="D60" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E60" t="s">
         <v>48</v>
       </c>
       <c r="I60" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K60">
         <v>7.5</v>
@@ -4549,19 +4546,19 @@
     </row>
     <row r="61" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B61">
         <v>114</v>
       </c>
       <c r="D61" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E61" t="s">
         <v>48</v>
       </c>
       <c r="I61" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K61">
         <v>7.5</v>
@@ -4582,19 +4579,19 @@
     </row>
     <row r="62" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B62">
         <v>114</v>
       </c>
       <c r="D62" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E62" t="s">
         <v>48</v>
       </c>
       <c r="I62" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K62">
         <v>7.5</v>
@@ -4615,19 +4612,19 @@
     </row>
     <row r="63" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B63">
         <v>114</v>
       </c>
       <c r="D63" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E63" t="s">
         <v>48</v>
       </c>
       <c r="I63" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K63">
         <v>7.5</v>
@@ -4648,19 +4645,19 @@
     </row>
     <row r="64" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B64">
         <v>114</v>
       </c>
       <c r="D64" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E64" t="s">
         <v>48</v>
       </c>
       <c r="I64" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K64">
         <v>7.5</v>
@@ -4681,19 +4678,19 @@
     </row>
     <row r="65" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B65">
         <v>114</v>
       </c>
       <c r="D65" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E65" t="s">
         <v>48</v>
       </c>
       <c r="I65" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K65">
         <v>7.5</v>
@@ -4714,19 +4711,19 @@
     </row>
     <row r="66" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B66">
         <v>114</v>
       </c>
       <c r="D66" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E66" t="s">
         <v>48</v>
       </c>
       <c r="I66" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K66">
         <v>7.5</v>
@@ -4747,19 +4744,19 @@
     </row>
     <row r="67" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B67">
         <v>114</v>
       </c>
       <c r="D67" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E67" t="s">
         <v>48</v>
       </c>
       <c r="I67" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K67">
         <v>7.5</v>
@@ -4780,19 +4777,19 @@
     </row>
     <row r="68" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B68">
         <v>114</v>
       </c>
       <c r="D68" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E68" t="s">
         <v>48</v>
       </c>
       <c r="I68" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K68">
         <v>7.5</v>
@@ -4813,19 +4810,19 @@
     </row>
     <row r="69" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B69">
         <v>114</v>
       </c>
       <c r="D69" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E69" t="s">
         <v>48</v>
       </c>
       <c r="I69" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K69">
         <v>7.5</v>
@@ -4846,19 +4843,19 @@
     </row>
     <row r="70" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B70">
         <v>114</v>
       </c>
       <c r="D70" t="s">
+        <v>56</v>
+      </c>
+      <c r="E70" t="s">
         <v>57</v>
       </c>
-      <c r="E70" t="s">
-        <v>58</v>
-      </c>
       <c r="I70" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K70">
         <v>7.9</v>
@@ -4878,19 +4875,19 @@
     </row>
     <row r="71" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B71">
         <v>114</v>
       </c>
       <c r="D71" t="s">
+        <v>56</v>
+      </c>
+      <c r="E71" t="s">
         <v>57</v>
       </c>
-      <c r="E71" t="s">
-        <v>58</v>
-      </c>
       <c r="I71" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K71">
         <v>7.9</v>
@@ -4910,19 +4907,19 @@
     </row>
     <row r="72" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B72">
         <v>114</v>
       </c>
       <c r="D72" t="s">
+        <v>56</v>
+      </c>
+      <c r="E72" t="s">
         <v>57</v>
       </c>
-      <c r="E72" t="s">
-        <v>58</v>
-      </c>
       <c r="I72" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K72">
         <v>7.9</v>
@@ -4942,19 +4939,19 @@
     </row>
     <row r="73" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B73">
         <v>114</v>
       </c>
       <c r="D73" t="s">
+        <v>56</v>
+      </c>
+      <c r="E73" t="s">
         <v>57</v>
       </c>
-      <c r="E73" t="s">
-        <v>58</v>
-      </c>
       <c r="I73" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K73">
         <v>7.9</v>
@@ -4974,19 +4971,19 @@
     </row>
     <row r="74" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B74">
         <v>114</v>
       </c>
       <c r="D74" t="s">
+        <v>56</v>
+      </c>
+      <c r="E74" t="s">
         <v>57</v>
       </c>
-      <c r="E74" t="s">
-        <v>58</v>
-      </c>
       <c r="I74" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K74">
         <v>7.9</v>
@@ -5006,19 +5003,19 @@
     </row>
     <row r="75" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B75">
         <v>114</v>
       </c>
       <c r="D75" t="s">
+        <v>56</v>
+      </c>
+      <c r="E75" t="s">
         <v>57</v>
       </c>
-      <c r="E75" t="s">
-        <v>58</v>
-      </c>
       <c r="I75" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K75">
         <v>7.9</v>
@@ -5038,19 +5035,19 @@
     </row>
     <row r="76" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B76">
         <v>114</v>
       </c>
       <c r="D76" t="s">
+        <v>56</v>
+      </c>
+      <c r="E76" t="s">
         <v>57</v>
       </c>
-      <c r="E76" t="s">
-        <v>58</v>
-      </c>
       <c r="I76" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K76">
         <v>7.9</v>
@@ -5070,19 +5067,19 @@
     </row>
     <row r="77" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B77">
         <v>114</v>
       </c>
       <c r="D77" t="s">
+        <v>56</v>
+      </c>
+      <c r="E77" t="s">
         <v>57</v>
       </c>
-      <c r="E77" t="s">
-        <v>58</v>
-      </c>
       <c r="I77" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K77">
         <v>7.9</v>
@@ -5102,19 +5099,19 @@
     </row>
     <row r="78" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B78">
         <v>114</v>
       </c>
       <c r="D78" t="s">
+        <v>56</v>
+      </c>
+      <c r="E78" t="s">
         <v>57</v>
       </c>
-      <c r="E78" t="s">
-        <v>58</v>
-      </c>
       <c r="I78" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K78">
         <v>7.9</v>
@@ -5134,19 +5131,19 @@
     </row>
     <row r="79" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B79">
         <v>114</v>
       </c>
       <c r="D79" t="s">
+        <v>56</v>
+      </c>
+      <c r="E79" t="s">
         <v>57</v>
       </c>
-      <c r="E79" t="s">
-        <v>58</v>
-      </c>
       <c r="I79" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K79">
         <v>7.9</v>
@@ -5166,19 +5163,19 @@
     </row>
     <row r="80" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B80">
         <v>114</v>
       </c>
       <c r="D80" t="s">
+        <v>56</v>
+      </c>
+      <c r="E80" t="s">
         <v>57</v>
       </c>
-      <c r="E80" t="s">
-        <v>58</v>
-      </c>
       <c r="I80" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K80">
         <v>7.9</v>
@@ -5198,19 +5195,19 @@
     </row>
     <row r="81" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B81">
         <v>114</v>
       </c>
       <c r="D81" t="s">
+        <v>56</v>
+      </c>
+      <c r="E81" t="s">
         <v>57</v>
       </c>
-      <c r="E81" t="s">
-        <v>58</v>
-      </c>
       <c r="I81" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K81">
         <v>7.9</v>
@@ -5230,19 +5227,19 @@
     </row>
     <row r="82" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B82">
         <v>114</v>
       </c>
       <c r="D82" t="s">
+        <v>56</v>
+      </c>
+      <c r="E82" t="s">
         <v>57</v>
       </c>
-      <c r="E82" t="s">
-        <v>58</v>
-      </c>
       <c r="I82" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K82">
         <v>7.9</v>
@@ -5262,19 +5259,19 @@
     </row>
     <row r="83" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B83">
         <v>114</v>
       </c>
       <c r="D83" t="s">
+        <v>56</v>
+      </c>
+      <c r="E83" t="s">
         <v>57</v>
       </c>
-      <c r="E83" t="s">
-        <v>58</v>
-      </c>
       <c r="I83" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K83">
         <v>7.9</v>
@@ -5294,19 +5291,19 @@
     </row>
     <row r="84" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B84">
         <v>114</v>
       </c>
       <c r="D84" t="s">
+        <v>56</v>
+      </c>
+      <c r="E84" t="s">
         <v>57</v>
       </c>
-      <c r="E84" t="s">
-        <v>58</v>
-      </c>
       <c r="I84" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K84">
         <v>7.9</v>
@@ -5326,19 +5323,19 @@
     </row>
     <row r="85" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B85">
         <v>114</v>
       </c>
       <c r="D85" t="s">
+        <v>56</v>
+      </c>
+      <c r="E85" t="s">
         <v>57</v>
       </c>
-      <c r="E85" t="s">
-        <v>58</v>
-      </c>
       <c r="I85" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K85">
         <v>7.9</v>
@@ -5358,19 +5355,19 @@
     </row>
     <row r="86" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B86">
         <v>114</v>
       </c>
       <c r="D86" t="s">
+        <v>56</v>
+      </c>
+      <c r="E86" t="s">
         <v>57</v>
       </c>
-      <c r="E86" t="s">
-        <v>58</v>
-      </c>
       <c r="I86" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K86">
         <v>7.9</v>
@@ -5390,19 +5387,19 @@
     </row>
     <row r="87" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B87">
         <v>114</v>
       </c>
       <c r="D87" t="s">
+        <v>56</v>
+      </c>
+      <c r="E87" t="s">
         <v>57</v>
       </c>
-      <c r="E87" t="s">
-        <v>58</v>
-      </c>
       <c r="I87" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K87">
         <v>7.9</v>
@@ -5422,19 +5419,19 @@
     </row>
     <row r="88" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B88">
         <v>114</v>
       </c>
       <c r="D88" t="s">
+        <v>56</v>
+      </c>
+      <c r="E88" t="s">
         <v>57</v>
       </c>
-      <c r="E88" t="s">
-        <v>58</v>
-      </c>
       <c r="I88" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K88">
         <v>7.9</v>
@@ -5454,19 +5451,19 @@
     </row>
     <row r="89" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B89">
         <v>114</v>
       </c>
       <c r="D89" t="s">
+        <v>56</v>
+      </c>
+      <c r="E89" t="s">
         <v>57</v>
       </c>
-      <c r="E89" t="s">
-        <v>58</v>
-      </c>
       <c r="I89" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K89">
         <v>7.9</v>
@@ -5486,19 +5483,19 @@
     </row>
     <row r="90" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B90">
         <v>115</v>
       </c>
       <c r="D90" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E90" t="s">
         <v>48</v>
       </c>
       <c r="I90" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K90">
         <v>7.4</v>
@@ -5518,19 +5515,19 @@
     </row>
     <row r="91" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B91">
         <v>115</v>
       </c>
       <c r="D91" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E91" t="s">
         <v>48</v>
       </c>
       <c r="I91" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K91">
         <v>7.4</v>
@@ -5550,19 +5547,19 @@
     </row>
     <row r="92" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B92">
         <v>115</v>
       </c>
       <c r="D92" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E92" t="s">
         <v>48</v>
       </c>
       <c r="I92" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K92">
         <v>7.3</v>
@@ -5582,19 +5579,19 @@
     </row>
     <row r="93" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B93">
         <v>115</v>
       </c>
       <c r="D93" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E93" t="s">
         <v>48</v>
       </c>
       <c r="I93" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K93">
         <v>7.3</v>
@@ -5764,10 +5761,10 @@
         <v>24</v>
       </c>
       <c r="V3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="W3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="X3" t="s">
         <v>25</v>
@@ -5838,10 +5835,10 @@
         <v>44</v>
       </c>
       <c r="V4" t="s">
+        <v>83</v>
+      </c>
+      <c r="W4" t="s">
         <v>84</v>
-      </c>
-      <c r="W4" t="s">
-        <v>85</v>
       </c>
       <c r="X4" t="s">
         <v>45</v>
@@ -5849,7 +5846,7 @@
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>